<commit_message>
Direct Write Excel for QC-16 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-16.xlsx
+++ b/FM-MN-07_QC-16.xlsx
@@ -1746,7 +1746,11 @@
       <c r="E6" s="23" t="inlineStr"/>
       <c r="F6" s="23" t="inlineStr"/>
       <c r="G6" s="23" t="inlineStr"/>
-      <c r="H6" s="23" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="23" t="inlineStr"/>
       <c r="J6" s="23" t="inlineStr"/>
       <c r="K6" s="23" t="inlineStr"/>
@@ -1787,7 +1791,11 @@
       <c r="E7" s="23" t="inlineStr"/>
       <c r="F7" s="23" t="inlineStr"/>
       <c r="G7" s="23" t="inlineStr"/>
-      <c r="H7" s="23" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="23" t="inlineStr"/>
       <c r="J7" s="23" t="inlineStr"/>
       <c r="K7" s="23" t="inlineStr"/>
@@ -1828,7 +1836,11 @@
       <c r="E8" s="23" t="inlineStr"/>
       <c r="F8" s="23" t="inlineStr"/>
       <c r="G8" s="23" t="inlineStr"/>
-      <c r="H8" s="23" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="23" t="inlineStr"/>
       <c r="J8" s="23" t="inlineStr"/>
       <c r="K8" s="23" t="inlineStr"/>
@@ -1869,7 +1881,11 @@
       <c r="E9" s="23" t="inlineStr"/>
       <c r="F9" s="23" t="inlineStr"/>
       <c r="G9" s="23" t="inlineStr"/>
-      <c r="H9" s="23" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="23" t="inlineStr"/>
       <c r="J9" s="23" t="inlineStr"/>
       <c r="K9" s="23" t="inlineStr"/>
@@ -1910,7 +1926,11 @@
       <c r="E10" s="23" t="inlineStr"/>
       <c r="F10" s="23" t="inlineStr"/>
       <c r="G10" s="23" t="inlineStr"/>
-      <c r="H10" s="23" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="23" t="inlineStr"/>
       <c r="J10" s="23" t="inlineStr"/>
       <c r="K10" s="23" t="inlineStr"/>
@@ -1945,7 +1965,11 @@
       <c r="E11" s="38" t="inlineStr"/>
       <c r="F11" s="38" t="inlineStr"/>
       <c r="G11" s="38" t="inlineStr"/>
-      <c r="H11" s="38" t="inlineStr"/>
+      <c r="H11" s="40" t="inlineStr">
+        <is>
+          <t>สายันต์</t>
+        </is>
+      </c>
       <c r="I11" s="38" t="inlineStr"/>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
@@ -2128,8 +2152,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-16 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-16.xlsx
+++ b/FM-MN-07_QC-16.xlsx
@@ -1754,7 +1754,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr"/>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="23" t="inlineStr"/>
       <c r="K6" s="23" t="inlineStr"/>
       <c r="L6" s="23" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr"/>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="23" t="inlineStr"/>
       <c r="K7" s="23" t="inlineStr"/>
       <c r="L7" s="23" t="inlineStr"/>
@@ -1844,7 +1852,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr"/>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="23" t="inlineStr"/>
       <c r="K8" s="23" t="inlineStr"/>
       <c r="L8" s="23" t="inlineStr"/>
@@ -1889,7 +1901,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="23" t="inlineStr"/>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="23" t="inlineStr"/>
       <c r="K9" s="23" t="inlineStr"/>
       <c r="L9" s="23" t="inlineStr"/>
@@ -1934,7 +1950,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="23" t="inlineStr"/>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="23" t="inlineStr"/>
       <c r="K10" s="23" t="inlineStr"/>
       <c r="L10" s="23" t="inlineStr"/>
@@ -1973,7 +1993,11 @@
           <t>สายันต์</t>
         </is>
       </c>
-      <c r="I11" s="38" t="inlineStr"/>
+      <c r="I11" s="40" t="inlineStr">
+        <is>
+          <t>สายันต์</t>
+        </is>
+      </c>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
       <c r="L11" s="38" t="inlineStr"/>
@@ -2159,8 +2183,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-16 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-16.xlsx
+++ b/FM-MN-07_QC-16.xlsx
@@ -1759,7 +1759,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="23" t="inlineStr"/>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="23" t="inlineStr"/>
       <c r="L6" s="23" t="inlineStr"/>
       <c r="M6" s="23" t="inlineStr"/>
@@ -1808,7 +1812,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="23" t="inlineStr"/>
+      <c r="J7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="23" t="inlineStr"/>
       <c r="L7" s="23" t="inlineStr"/>
       <c r="M7" s="23" t="inlineStr"/>
@@ -1857,7 +1865,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="23" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="23" t="inlineStr"/>
       <c r="L8" s="23" t="inlineStr"/>
       <c r="M8" s="23" t="inlineStr"/>
@@ -1906,7 +1918,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="23" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="23" t="inlineStr"/>
       <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="23" t="inlineStr"/>
@@ -1955,7 +1971,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="23" t="inlineStr"/>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="23" t="inlineStr"/>
       <c r="L10" s="23" t="inlineStr"/>
       <c r="M10" s="23" t="inlineStr"/>
@@ -1998,7 +2018,11 @@
           <t>สายันต์</t>
         </is>
       </c>
-      <c r="J11" s="38" t="inlineStr"/>
+      <c r="J11" s="40" t="inlineStr">
+        <is>
+          <t>สายันต์</t>
+        </is>
+      </c>
       <c r="K11" s="38" t="inlineStr"/>
       <c r="L11" s="38" t="inlineStr"/>
       <c r="M11" s="38" t="inlineStr"/>
@@ -2183,8 +2207,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-16 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-16.xlsx
+++ b/FM-MN-07_QC-16.xlsx
@@ -1765,7 +1765,11 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="23" t="inlineStr"/>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="23" t="inlineStr"/>
       <c r="N6" s="23" t="inlineStr"/>
       <c r="O6" s="23" t="inlineStr"/>
@@ -1818,7 +1822,11 @@
         </is>
       </c>
       <c r="K7" s="23" t="inlineStr"/>
-      <c r="L7" s="23" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="23" t="inlineStr"/>
       <c r="N7" s="23" t="inlineStr"/>
       <c r="O7" s="23" t="inlineStr"/>
@@ -1871,7 +1879,11 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="23" t="inlineStr"/>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="23" t="inlineStr"/>
       <c r="N8" s="23" t="inlineStr"/>
       <c r="O8" s="23" t="inlineStr"/>
@@ -1924,7 +1936,11 @@
         </is>
       </c>
       <c r="K9" s="23" t="inlineStr"/>
-      <c r="L9" s="23" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="23" t="inlineStr"/>
       <c r="N9" s="23" t="inlineStr"/>
       <c r="O9" s="23" t="inlineStr"/>
@@ -1977,7 +1993,11 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="23" t="inlineStr"/>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="23" t="inlineStr"/>
       <c r="N10" s="23" t="inlineStr"/>
       <c r="O10" s="23" t="inlineStr"/>
@@ -2024,7 +2044,11 @@
         </is>
       </c>
       <c r="K11" s="38" t="inlineStr"/>
-      <c r="L11" s="38" t="inlineStr"/>
+      <c r="L11" s="40" t="inlineStr">
+        <is>
+          <t>สายันต์</t>
+        </is>
+      </c>
       <c r="M11" s="38" t="inlineStr"/>
       <c r="N11" s="38" t="inlineStr"/>
       <c r="O11" s="38" t="inlineStr"/>
@@ -2207,8 +2231,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>